<commit_message>
docs(admissions): register sync — SPRINT-06/NEW-18 closure (admission funnel)
BOOK-21 bumped to v0.2 (full funnel -> exists; C21.5 eval-harness gate,
full GPS Pareto orientation, program fee data, onboarding-journey/G16
credit_pre_evaluations hand-offs all named as explicit remaining gaps).
TRACEABILITY G17 += NEW-18 (C21.1-C21.4 verified, E2E DoD fixture
passing). CHANGELOG entry. BACKLOG_TARGET.xlsx: BLG-022..031 updated
(028/029 orientation-adjacent items left "In corso" — GPS/cost
projection honestly incomplete, not silently marked done).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TARGET.xlsx
+++ b/BACKLOG_TARGET.xlsx
@@ -2125,10 +2125,14 @@
       </c>
       <c r="M23" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N23" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>admission_intakes + admission_requirements (admission_service.py). Requisiti versionati per intake, immutabili dopo l'apertura (BOOK-21 §3, enforced a livello servizio).</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="23.85" customHeight="1" s="13">
       <c r="A24" s="15" t="inlineStr">
@@ -2193,10 +2197,14 @@
       </c>
       <c r="M24" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N24" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N24" s="16" t="inlineStr">
+        <is>
+          <t>admission_applications, state machine a 11 stati (BOOK-21 §4) + qualification_documents per i documenti allegati.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="23.85" customHeight="1" s="13">
       <c r="A25" s="15" t="inlineStr">
@@ -2261,10 +2269,14 @@
       </c>
       <c r="M25" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N25" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N25" s="16" t="inlineStr">
+        <is>
+          <t>lead_conversion_service.convert_crm_lead_to_application legge CRMLeadMapping direttamente (non tramite crm.py, mai montato). Gap onesto: nessun campo nome/email reale raggiungibile da CRMLeadMapping — applicant_data popolato solo con campi reali (lead_score, sync_status), mai inventato.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="23.85" customHeight="1" s="13">
       <c r="A26" s="15" t="inlineStr">
@@ -2329,10 +2341,14 @@
       </c>
       <c r="M26" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N26" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N26" s="16" t="inlineStr">
+        <is>
+          <t>issue_offer (C21.2: richiede verdetto eligible/conditional) + accept_offer/decline_offer/expire_offer, admission_service.py.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="23.85" customHeight="1" s="13">
       <c r="A27" s="15" t="inlineStr">
@@ -2397,10 +2413,14 @@
       </c>
       <c r="M27" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N27" s="16" t="n"/>
+          <t>In corso</t>
+        </is>
+      </c>
+      <c r="N27" s="16" t="inlineStr">
+        <is>
+          <t>Anteprima crediti riconoscibili reale (riusa preval_workflow_service.compute_instant_estimate, zero-persistenza). La componente GPS/percorso (scenari Pareto multi-obiettivo) NON implementata: il motore GPS richiede un gemello reale, che non esiste pre-immatricolazione — tensione architetturale onestamente disclosurata in BOOK-21 v0.2, non un semplice rinvio.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="23.85" customHeight="1" s="13">
       <c r="A28" s="15" t="inlineStr">
@@ -2465,10 +2485,14 @@
       </c>
       <c r="M28" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N28" s="16" t="n"/>
+          <t>In corso</t>
+        </is>
+      </c>
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>ETA: stima standalone semplice (CFU residui / 60 CFU/anno). Costo: placeholder onesto null — nessun campo fee/retta esiste ancora su Program. Nessun confronto multi-scenario Pareto-completo.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="23.85" customHeight="1" s="13">
       <c r="A29" s="15" t="inlineStr">
@@ -2533,10 +2557,14 @@
       </c>
       <c r="M29" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N29" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N29" s="16" t="inlineStr">
+        <is>
+          <t>qualification_service.add_qualification + add_qualification_document (stessa convenzione document_type/storage_uri di PrevalDocument).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="23.85" customHeight="1" s="13">
       <c r="A30" s="15" t="inlineStr">
@@ -2601,10 +2629,14 @@
       </c>
       <c r="M30" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N30" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N30" s="16" t="inlineStr">
+        <is>
+          <t>run_tier1_evaluation. Matching istituzione: euristica onestamente disclosurata (match esatto poi substring case-insensitive su external_courses.source_institution_name) — nessuna vera politica DM 931/2024 codificata, nessun matching fabbricato quando non esiste corrispondenza.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="23.85" customHeight="1" s="13">
       <c r="A31" s="15" t="inlineStr">
@@ -2669,10 +2701,14 @@
       </c>
       <c r="M31" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N31" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N31" s="16" t="inlineStr">
+        <is>
+          <t>escalate_evaluation_tier (tier 'assisted'/'committee'), motivo obbligatorio non-vuoto (R21.1).</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="23.85" customHeight="1" s="13">
       <c r="A32" s="15" t="inlineStr">
@@ -2737,10 +2773,14 @@
       </c>
       <c r="M32" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N32" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N32" s="16" t="inlineStr">
+        <is>
+          <t>decide_eligibility + eligibility_verdicts. R21.2 (unmet_requirements obbligatorio per verdetti negativi/condizionati) + R21.3 (admissions_officer+ per verdetto negativo) entrambi verificati con property/fixture test.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="23.85" customHeight="1" s="13">
       <c r="A33" s="15" t="inlineStr">

</xml_diff>

<commit_message>
docs(preval): register sync — SPRINT-07/NEW-17d closure (golden set + eval gate)
BOOK-21A bumped to v0.3 (F4 -> exists; C21A.6 closed, C21A.7 real and
CI-wired; certification honestly provisional -- zero real historical
data in this environment). TRACEABILITY G17 += NEW-17d. CHANGELOG entry
including the honest M1-milestone framing (functionally complete, but
BACKLOG_TARGET.xlsx's own bookkeeping still shows 17 stale rows from a
now-3x-confirmed pre-existing doc-sync gap in SPRINT-02/03/04/06 -- not
backfilled here, out of scope, flagged more strongly this time given
the repeated recurrence). BACKLOG_TARGET.xlsx: BLG-032 -> Fatto.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TARGET.xlsx
+++ b/BACKLOG_TARGET.xlsx
@@ -2845,10 +2845,14 @@
       </c>
       <c r="M33" s="16" t="inlineStr">
         <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="N33" s="16" t="n"/>
+          <t>Fatto</t>
+        </is>
+      </c>
+      <c r="N33" s="16" t="inlineStr">
+        <is>
+          <t>Golden set (preval_eval_builder.py) + metriche (preval_eval_metrics.py: accuracy CFU, precision/recall, escalation/override rate) + learning loop (override HITL -&gt; corretta riga -&gt; golden set aggiornato, chiude anche C21A.6) + gate CI reale (preval_eval_gate.py, blocca build immagine in build-push-images.yml) + report settimanale + config soglia auto-approvazione per-CDS (default OFF, mai attivata). Certificazione onestamente PROVVISORIA: zero dati storici reali in questo ambiente (confermato in pre-flight) — golden set bootstrap (fixture Conti + traffico reale sprint 02-06), non un corpus storico. VRA-exactness e accuracy per componente (estrazione/SSD) onestamente None — nessun ground truth esiste per misurarle.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="23.85" customHeight="1" s="13">
       <c r="A34" s="17" t="inlineStr">

</xml_diff>

<commit_message>
docs(BOOK-26): register sync — AVA-01…AVA-12 (G22 fully closed, 12-sprint program)
Adds BOOK-26 (Accreditation, Quality Assurance & DM 1154/2021 Compliance) and
syncs the masterbook apparatus (index, traceability G22, glossary, changelog)
plus both xlsx trackers for the 12-sprint AVA program delivered in
dlu_builder_tk: faculty-requirement engine, Art. 3/4 accreditation lifecycle,
Allegato E indicators, SUA-CdS/SMA/Riesame tracking, Auditor/CEV persona,
immutable evidence registry, alert engine, and Allegato C judgment workflow.

Also re-runs scripts/sync-masterbook.sh, which pulls in pre-existing mirror
drift in docs/masterbook/ unrelated to this program (BOOK-06/07/08/10A/10B/
11/16/17/19/20 mirrors were stale from earlier sprints whose sync never ran).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BACKLOG_TARGET.xlsx
+++ b/BACKLOG_TARGET.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N106"/>
+  <dimension ref="A1:N121"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="12" min="1" max="1"/>
@@ -7817,6 +7817,1011 @@
         </is>
       </c>
       <c r="N106" s="16" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="12" t="inlineStr">
+        <is>
+          <t>BLG-106</t>
+        </is>
+      </c>
+      <c r="B107" s="12" t="inlineStr">
+        <is>
+          <t>AVA-03</t>
+        </is>
+      </c>
+      <c r="C107" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D107" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E107" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="F107" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G107" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H107" s="12" t="inlineStr">
+        <is>
+          <t>Requisiti Docenza (Allegati A &amp; D)</t>
+        </is>
+      </c>
+      <c r="I107" s="12" t="inlineStr">
+        <is>
+          <t>Calcolo automatico Dtot/Ttot (docenti di riferimento richiesti vs disponibili, scalati per numerosità studenti)</t>
+        </is>
+      </c>
+      <c r="J107" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K107" s="12" t="inlineStr">
+        <is>
+          <t>Coordinatore CdS</t>
+        </is>
+      </c>
+      <c r="L107" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-03</t>
+        </is>
+      </c>
+      <c r="M107" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="12" t="inlineStr">
+        <is>
+          <t>BLG-107</t>
+        </is>
+      </c>
+      <c r="B108" s="12" t="inlineStr">
+        <is>
+          <t>AVA-02</t>
+        </is>
+      </c>
+      <c r="C108" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D108" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E108" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G108" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H108" s="12" t="inlineStr">
+        <is>
+          <t>Requisiti Docenza (Allegati A &amp; D)</t>
+        </is>
+      </c>
+      <c r="I108" s="12" t="inlineStr">
+        <is>
+          <t>Rule pack Allegato A (minimi per tipo corso/modalità) e numerosità Allegato D, versionati e governati</t>
+        </is>
+      </c>
+      <c r="J108" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K108" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L108" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-02</t>
+        </is>
+      </c>
+      <c r="M108" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="12" t="inlineStr">
+        <is>
+          <t>BLG-108</t>
+        </is>
+      </c>
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>AVA-04</t>
+        </is>
+      </c>
+      <c r="C109" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E109" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="F109" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G109" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H109" s="12" t="inlineStr">
+        <is>
+          <t>Registro Accreditamento (Art. 3-4)</t>
+        </is>
+      </c>
+      <c r="I109" s="12" t="inlineStr">
+        <is>
+          <t>Registro accreditamento sedi/corsi: stato, esito, scadenza, durata concessa</t>
+        </is>
+      </c>
+      <c r="J109" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K109" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L109" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-01/04</t>
+        </is>
+      </c>
+      <c r="M109" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="12" t="inlineStr">
+        <is>
+          <t>BLG-109</t>
+        </is>
+      </c>
+      <c r="B110" s="12" t="inlineStr">
+        <is>
+          <t>AVA-12</t>
+        </is>
+      </c>
+      <c r="C110" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D110" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E110" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F110" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G110" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H110" s="12" t="inlineStr">
+        <is>
+          <t>Registro Accreditamento (Art. 3-4)</t>
+        </is>
+      </c>
+      <c r="I110" s="12" t="inlineStr">
+        <is>
+          <t>Calcolo esito Art. 3 dalla distribuzione dei giudizi (pienamente soddisfacente/soddisfacente/condizionato/non soddisfacente)</t>
+        </is>
+      </c>
+      <c r="J110" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K110" s="12" t="inlineStr">
+        <is>
+          <t>CEV</t>
+        </is>
+      </c>
+      <c r="L110" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-04/12</t>
+        </is>
+      </c>
+      <c r="M110" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="12" t="inlineStr">
+        <is>
+          <t>BLG-110</t>
+        </is>
+      </c>
+      <c r="B111" s="12" t="inlineStr">
+        <is>
+          <t>AVA-04</t>
+        </is>
+      </c>
+      <c r="C111" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D111" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E111" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="F111" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G111" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H111" s="12" t="inlineStr">
+        <is>
+          <t>Registro Accreditamento (Art. 3-4)</t>
+        </is>
+      </c>
+      <c r="I111" s="12" t="inlineStr">
+        <is>
+          <t>Verifica decadenza automatica Art. 4 (mancata attivazione, sospensione biennale, verifica docenza 30/11, ISEF)</t>
+        </is>
+      </c>
+      <c r="J111" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K111" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L111" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-04</t>
+        </is>
+      </c>
+      <c r="M111" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="inlineStr">
+        <is>
+          <t>BLG-111</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>AVA-05</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D112" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E112" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G112" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H112" s="12" t="inlineStr">
+        <is>
+          <t>Indicatori Allegato E</t>
+        </is>
+      </c>
+      <c r="I112" s="12" t="inlineStr">
+        <is>
+          <t>Catalogo indicatori ministeriali per ambito A-E</t>
+        </is>
+      </c>
+      <c r="J112" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K112" s="12" t="inlineStr">
+        <is>
+          <t>NUV</t>
+        </is>
+      </c>
+      <c r="L112" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-05</t>
+        </is>
+      </c>
+      <c r="M112" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t>BLG-112</t>
+        </is>
+      </c>
+      <c r="B113" s="12" t="inlineStr">
+        <is>
+          <t>AVA-06</t>
+        </is>
+      </c>
+      <c r="C113" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E113" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G113" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H113" s="12" t="inlineStr">
+        <is>
+          <t>Indicatori Allegato E</t>
+        </is>
+      </c>
+      <c r="I113" s="12" t="inlineStr">
+        <is>
+          <t>Calcolo automatico degli indicatori disponibili (% ore docenza t.i., % CFU I anno) da dati reali di corso/docenza</t>
+        </is>
+      </c>
+      <c r="J113" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K113" s="12" t="inlineStr">
+        <is>
+          <t>Coordinatore CdS</t>
+        </is>
+      </c>
+      <c r="L113" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-06</t>
+        </is>
+      </c>
+      <c r="M113" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t>BLG-113</t>
+        </is>
+      </c>
+      <c r="B114" s="12" t="inlineStr">
+        <is>
+          <t>AVA-07</t>
+        </is>
+      </c>
+      <c r="C114" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D114" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E114" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G114" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H114" s="12" t="inlineStr">
+        <is>
+          <t>SUA-CdS, SMA &amp; Riesame Ciclico</t>
+        </is>
+      </c>
+      <c r="I114" s="12" t="inlineStr">
+        <is>
+          <t>Tracciamento completezza SUA-CdS (sezioni Amministrazione/Qualità) e scadenzario</t>
+        </is>
+      </c>
+      <c r="J114" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K114" s="12" t="inlineStr">
+        <is>
+          <t>Coordinatore CdS</t>
+        </is>
+      </c>
+      <c r="L114" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-07</t>
+        </is>
+      </c>
+      <c r="M114" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="12" t="inlineStr">
+        <is>
+          <t>BLG-114</t>
+        </is>
+      </c>
+      <c r="B115" s="12" t="inlineStr">
+        <is>
+          <t>AVA-07</t>
+        </is>
+      </c>
+      <c r="C115" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E115" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="F115" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G115" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H115" s="12" t="inlineStr">
+        <is>
+          <t>SUA-CdS, SMA &amp; Riesame Ciclico</t>
+        </is>
+      </c>
+      <c r="I115" s="12" t="inlineStr">
+        <is>
+          <t>Gestione SMA e Riesame Ciclico con azioni di miglioramento collegate</t>
+        </is>
+      </c>
+      <c r="J115" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K115" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L115" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-07</t>
+        </is>
+      </c>
+      <c r="M115" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>BLG-115</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t>AVA-08</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D116" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E116" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G116" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H116" s="12" t="inlineStr">
+        <is>
+          <t>Persona Auditor &amp; CEV</t>
+        </is>
+      </c>
+      <c r="I116" s="12" t="inlineStr">
+        <is>
+          <t>Accesso esterno Auditor MUR/ANVUR/CEV: concessioni con scope e validità temporale, watermark, audit trail</t>
+        </is>
+      </c>
+      <c r="J116" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K116" s="12" t="inlineStr">
+        <is>
+          <t>System Admin</t>
+        </is>
+      </c>
+      <c r="L116" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-08</t>
+        </is>
+      </c>
+      <c r="M116" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="12" t="inlineStr">
+        <is>
+          <t>BLG-116</t>
+        </is>
+      </c>
+      <c r="B117" s="12" t="inlineStr">
+        <is>
+          <t>AVA-10</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D117" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E117" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F117" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G117" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H117" s="12" t="inlineStr">
+        <is>
+          <t>Persona Auditor &amp; CEV</t>
+        </is>
+      </c>
+      <c r="I117" s="12" t="inlineStr">
+        <is>
+          <t>Fascicolo di sede/corso per la CEV: punti di attenzione, evidenze collegate, giudizio a 4 fasce</t>
+        </is>
+      </c>
+      <c r="J117" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K117" s="12" t="inlineStr">
+        <is>
+          <t>CEV</t>
+        </is>
+      </c>
+      <c r="L117" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-10/12</t>
+        </is>
+      </c>
+      <c r="M117" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t>BLG-117</t>
+        </is>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>AVA-09</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G118" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H118" s="12" t="inlineStr">
+        <is>
+          <t>Evidenze &amp; Snapshot</t>
+        </is>
+      </c>
+      <c r="I118" s="12" t="inlineStr">
+        <is>
+          <t>Registro evidenze collegate a indicatori e punti di attenzione, con provenienza dati</t>
+        </is>
+      </c>
+      <c r="J118" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K118" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L118" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-09</t>
+        </is>
+      </c>
+      <c r="M118" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
+        <is>
+          <t>BLG-118</t>
+        </is>
+      </c>
+      <c r="B119" s="12" t="inlineStr">
+        <is>
+          <t>AVA-09</t>
+        </is>
+      </c>
+      <c r="C119" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D119" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E119" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F119" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G119" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H119" s="12" t="inlineStr">
+        <is>
+          <t>Evidenze &amp; Snapshot</t>
+        </is>
+      </c>
+      <c r="I119" s="12" t="inlineStr">
+        <is>
+          <t>Snapshot cruscotto immutabili e datati, con firma opzionale</t>
+        </is>
+      </c>
+      <c r="J119" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K119" s="12" t="inlineStr">
+        <is>
+          <t>Auditor</t>
+        </is>
+      </c>
+      <c r="L119" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-09</t>
+        </is>
+      </c>
+      <c r="M119" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="12" t="inlineStr">
+        <is>
+          <t>BLG-119</t>
+        </is>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>AVA-11</t>
+        </is>
+      </c>
+      <c r="C120" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G120" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H120" s="12" t="inlineStr">
+        <is>
+          <t>Alert &amp; Cruscotti</t>
+        </is>
+      </c>
+      <c r="I120" s="12" t="inlineStr">
+        <is>
+          <t>Motore di alert/early-warning (10 codici del catalogo §7, severità, destinatari per ruolo)</t>
+        </is>
+      </c>
+      <c r="J120" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K120" s="12" t="inlineStr">
+        <is>
+          <t>PQA</t>
+        </is>
+      </c>
+      <c r="L120" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-11</t>
+        </is>
+      </c>
+      <c r="M120" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="12" t="inlineStr">
+        <is>
+          <t>BLG-120</t>
+        </is>
+      </c>
+      <c r="B121" s="12" t="inlineStr">
+        <is>
+          <t>AVA-10</t>
+        </is>
+      </c>
+      <c r="C121" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="D121" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="E121" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="F121" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="G121" s="12" t="inlineStr">
+        <is>
+          <t>26. Accreditamento &amp; Assicurazione Qualità (DM 1154/2021)</t>
+        </is>
+      </c>
+      <c r="H121" s="12" t="inlineStr">
+        <is>
+          <t>Alert &amp; Cruscotti</t>
+        </is>
+      </c>
+      <c r="I121" s="12" t="inlineStr">
+        <is>
+          <t>Cruscotti dedicati Auditor, PQA/NUV, Coordinatore CdS</t>
+        </is>
+      </c>
+      <c r="J121" s="12" t="inlineStr">
+        <is>
+          <t>Nuova</t>
+        </is>
+      </c>
+      <c r="K121" s="12" t="inlineStr">
+        <is>
+          <t>Auditor</t>
+        </is>
+      </c>
+      <c r="L121" s="12" t="inlineStr">
+        <is>
+          <t>T14 · AVA-10</t>
+        </is>
+      </c>
+      <c r="M121" s="12" t="inlineStr">
+        <is>
+          <t>Fatto</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N106"/>
@@ -7838,7 +8843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="12" min="1" max="1"/>
@@ -8751,25 +9756,493 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="13">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>AVA-01</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F24" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A24,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H24" s="12">
+        <f>IF(F24=0,"—",G24/F24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>AVA-02</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F25" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A25)</f>
+        <v/>
+      </c>
+      <c r="G25" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A25,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H25" s="12">
+        <f>IF(F25=0,"—",G25/F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>AVA-03</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F26" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A26)</f>
+        <v/>
+      </c>
+      <c r="G26" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A26,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H26" s="12">
+        <f>IF(F26=0,"—",G26/F26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>AVA-04</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F27" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A27)</f>
+        <v/>
+      </c>
+      <c r="G27" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A27,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H27" s="12">
+        <f>IF(F27=0,"—",G27/F27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>AVA-05</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F28" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A28)</f>
+        <v/>
+      </c>
+      <c r="G28" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A28,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H28" s="12">
+        <f>IF(F28=0,"—",G28/F28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>AVA-06</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F29" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A29)</f>
+        <v/>
+      </c>
+      <c r="G29" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A29,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H29" s="12">
+        <f>IF(F29=0,"—",G29/F29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>AVA-07</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F30" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A30)</f>
+        <v/>
+      </c>
+      <c r="G30" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A30,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H30" s="12">
+        <f>IF(F30=0,"—",G30/F30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>AVA-08</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F31" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A31)</f>
+        <v/>
+      </c>
+      <c r="G31" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A31,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H31" s="12">
+        <f>IF(F31=0,"—",G31/F31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>AVA-09</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F32" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A32)</f>
+        <v/>
+      </c>
+      <c r="G32" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A32,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H32" s="12">
+        <f>IF(F32=0,"—",G32/F32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>AVA-10</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F33" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A33)</f>
+        <v/>
+      </c>
+      <c r="G33" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A33,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H33" s="12">
+        <f>IF(F33=0,"—",G33/F33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>AVA-11</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F34" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A34)</f>
+        <v/>
+      </c>
+      <c r="G34" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A34,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H34" s="12">
+        <f>IF(F34=0,"—",G34/F34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>AVA-12</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>A+B</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="F35" s="12">
+        <f>COUNTIF('Backlog Target'!$B$2:$B$200,A35)</f>
+        <v/>
+      </c>
+      <c r="G35" s="12">
+        <f>COUNTIFS('Backlog Target'!$B$2:$B$200,A35,'Backlog Target'!$M$2:$M$200,"Fatto")</f>
+        <v/>
+      </c>
+      <c r="H35" s="12">
+        <f>IF(F35=0,"—",G35/F35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>TOTALE</t>
         </is>
       </c>
-      <c r="B24" s="23" t="n"/>
-      <c r="C24" s="23" t="n"/>
-      <c r="D24" s="23" t="n"/>
-      <c r="E24" s="23" t="n"/>
-      <c r="F24" s="23">
-        <f>SUM(F2:F23)</f>
-        <v/>
-      </c>
-      <c r="G24" s="23">
-        <f>SUM(G2:G23)</f>
-        <v/>
-      </c>
-      <c r="H24" s="24">
-        <f>IF(F24=0,0,G24/F24)</f>
+      <c r="B36" s="23" t="n"/>
+      <c r="C36" s="23" t="n"/>
+      <c r="D36" s="23" t="n"/>
+      <c r="E36" s="23" t="n"/>
+      <c r="F36" s="23">
+        <f>SUM(F2:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="23">
+        <f>SUM(G2:G35)</f>
+        <v/>
+      </c>
+      <c r="H36" s="24">
+        <f>IF(F36=0,0,G36/F36)</f>
         <v/>
       </c>
     </row>
@@ -8825,7 +10298,7 @@
       </c>
       <c r="B3" s="21" t="inlineStr">
         <is>
-          <t>Card NEW-xx del PIANO_SPRINT_TARGET.md (numerazione registro masterbook)</t>
+          <t>Card NEW-xx del PIANO_SPRINT_TARGET.md (numerazione registro masterbook) o AVA-xx (programma DM 1154/2021, TRACEABILITY.md G22, fuori dal piano NEW-xx originale)</t>
         </is>
       </c>
     </row>
@@ -8837,7 +10310,7 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>Ondata W0–W4 · squad A (Platform) / B (AI &amp; Product) · sprint di calendario S1–S11 da set 2026</t>
+          <t>Ondata W0–W4 (piano NEW-xx originale) + W5 (programma AVA, post-piano) · squad A (Platform) / B (AI &amp; Product) / A+B · sprint di calendario S1–S22c (piano originale), S23–S25 (AVA, disclosed placement — nessun piano preesistente assegnava AVA a un'ondata/sprint-cal.)</t>
         </is>
       </c>
     </row>
@@ -8849,7 +10322,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>M1 PreEval+Intake (fine nov 2026) · M2 Faculty+Student loop (fine dic 2026) · M3 target completo (metà feb 2027)</t>
+          <t>M1 PreEval+Intake (fine nov 2026) · M2 Faculty+Student loop (fine dic 2026) · M3 target completo (metà feb 2027) · M4 Accreditamento &amp; QA — DM 1154/2021 (fuori scope piano originale, aggiunta AVA)</t>
         </is>
       </c>
     </row>
@@ -8861,7 +10334,7 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t>Nuova (75) o Estensione (7) — da ALBERO_FUNZIONALITA_TARGET.xlsx</t>
+          <t>Nuova (90 = 75 piano originale + 15 AVA) o Estensione (7) — da ALBERO_FUNZIONALITA_TARGET.xlsx</t>
         </is>
       </c>
     </row>
@@ -8885,7 +10358,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>NEW-17f (fondazioni) e NEW-29 includono anche lavoro non-feature (migrazioni, taxonomy, conformance): qui compaiono solo le feature dell albero</t>
+          <t>NEW-17f (fondazioni) e NEW-29 includono anche lavoro non-feature (migrazioni, taxonomy, conformance): qui compaiono solo le feature dell albero. AVA-01 (schema-only) segue la stessa convenzione — zero righe qui, coerente con zero righe proprie nell'Albero.</t>
         </is>
       </c>
     </row>

</xml_diff>